<commit_message>
fixed Source column value in consolidated_report.xlsx
</commit_message>
<xml_diff>
--- a/data/subsidiaries/parent_co.xlsx
+++ b/data/subsidiaries/parent_co.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00-CLaude-Plugins\financial-consolidation\data\subsidiaries\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00-CLaude-Plugins\fin-consol-auto-populate\data\subsidiaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDED1F7-07AD-4C4D-BE07-9E85219D157A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7536FC37-827D-45A4-AE2A-23BC46A6CA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="3060" windowWidth="15480" windowHeight="10785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5220" yWindow="5910" windowWidth="13245" windowHeight="9045" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,14 @@
     <sheet name="CF" sheetId="3" r:id="rId3"/>
     <sheet name="EQ" sheetId="4" r:id="rId4"/>
     <sheet name="META" sheetId="5" r:id="rId5"/>
+    <sheet name="ICO" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="75">
   <si>
     <t>account_code</t>
   </si>
@@ -219,6 +220,36 @@
   </si>
   <si>
     <t>ownership_pct</t>
+  </si>
+  <si>
+    <t>account_no</t>
+  </si>
+  <si>
+    <t>to_party</t>
+  </si>
+  <si>
+    <t>account_type</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Sub SGD</t>
+  </si>
+  <si>
+    <t>Trade Receivable</t>
+  </si>
+  <si>
+    <t>SGD</t>
+  </si>
+  <si>
+    <t>Q4 goods</t>
+  </si>
+  <si>
+    <t>IC Loan</t>
+  </si>
+  <si>
+    <t>Facility drawdown</t>
   </si>
 </sst>
 </file>
@@ -702,10 +733,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1012,4 +1039,74 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2">
+        <v>50000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3">
+        <v>100000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
saved Excel data files
</commit_message>
<xml_diff>
--- a/data/subsidiaries/parent_co.xlsx
+++ b/data/subsidiaries/parent_co.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\00-CLaude-Plugins\fin-consol-auto-populate\data\subsidiaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7536FC37-827D-45A4-AE2A-23BC46A6CA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{360AE858-EAC0-4B69-A31F-5A885537568B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5220" yWindow="5910" windowWidth="13245" windowHeight="9045" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12705" yWindow="6345" windowWidth="13245" windowHeight="9045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS" sheetId="1" r:id="rId1"/>
@@ -929,6 +929,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -995,6 +1000,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1045,6 +1053,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>